<commit_message>
Transfer of progress within data lab to outside data lab v0.2 to v0.7
</commit_message>
<xml_diff>
--- a/inst/extdata/examples/confidential_control_file_w_metadata/control_file.xlsx
+++ b/inst/extdata/examples/confidential_control_file_w_metadata/control_file.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NotBackedUp\Analytic_tool_building\IDIr\inst\extdata\examples\confidential_control_file_w_metadata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\MAA2023-46\projects\Tool development\IDIr\inst\extdata\examples\confidential_control_file_w_metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6B04B41F-DD22-4E41-9678-1D7D00200718}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{470C36D5-54F7-4DBC-9CCD-3C21652A0C6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{22CB9F0F-9B95-4F37-9549-688E39B26EC5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{22CB9F0F-9B95-4F37-9549-688E39B26EC5}"/>
   </bookViews>
   <sheets>
     <sheet name="metadata" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="71">
   <si>
     <t>COMMAND</t>
   </si>
@@ -222,17 +222,41 @@
     <t>CHANGES</t>
   </si>
   <si>
-    <t>This column requires random rounding (RR3), and suppression against three different columns.</t>
-  </si>
-  <si>
     <t>This column requires graduate random rounding (GRR), and suppression against three different columns.</t>
+  </si>
+  <si>
+    <t>SEED</t>
+  </si>
+  <si>
+    <t>seed_col</t>
+  </si>
+  <si>
+    <t>This column requires random rounding (RR3), and suppression against three different columns. A seed column is provided to enforce consistent random rounding.</t>
+  </si>
+  <si>
+    <t>This column has been generated to ensure that identical groups of people are always randomly rounded in the same way. It is dropped as it is not needed in the final output.</t>
+  </si>
+  <si>
+    <t>Random rounding &amp; seeds:</t>
+  </si>
+  <si>
+    <t>The microdata output guide requires that identical groups of people are randomly rounded in identical ways.</t>
+  </si>
+  <si>
+    <t>This can be done via providing a seed column. Where the seed is identical random rounding will also be identical.</t>
+  </si>
+  <si>
+    <t>The summary tool provides a SEED option designed for making this seed column.</t>
+  </si>
+  <si>
+    <t>If no seed column is provided, the tool will use the 'stable_above' option to enforce some consistent rounding.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -245,6 +269,12 @@
       <color theme="1"/>
       <name val="Arial Mäori"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial Mäori"/>
     </font>
   </fonts>
   <fills count="2">
@@ -267,10 +297,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -289,9 +320,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -329,7 +360,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -435,7 +466,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -577,7 +608,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -585,62 +616,62 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EBE5773-DF1B-4A7E-AC76-C5025400B8B9}">
-  <dimension ref="A1:B23"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:B32"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="12.5" customWidth="1"/>
     <col min="2" max="2" width="15.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="15">
       <c r="A1" s="1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="15">
       <c r="A3" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2">
       <c r="A4" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ht="15">
       <c r="A5" s="1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2">
       <c r="A6" s="2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" ht="15">
       <c r="A7" s="1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2">
       <c r="A8" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" ht="15">
       <c r="A11" s="1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" ht="15">
       <c r="A12" s="1"/>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2">
       <c r="A13" t="s">
         <v>59</v>
       </c>
@@ -648,7 +679,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2">
       <c r="A14" t="s">
         <v>1</v>
       </c>
@@ -656,7 +687,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:2">
       <c r="A15" t="s">
         <v>50</v>
       </c>
@@ -664,7 +695,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:2">
       <c r="A16" t="s">
         <v>51</v>
       </c>
@@ -672,7 +703,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2">
       <c r="A17" t="s">
         <v>52</v>
       </c>
@@ -680,23 +711,23 @@
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2">
       <c r="A18" t="s">
         <v>8</v>
       </c>
       <c r="B18" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
       <c r="A19" t="s">
         <v>9</v>
       </c>
       <c r="B19" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
       <c r="A20" t="s">
         <v>10</v>
       </c>
@@ -704,7 +735,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:2">
       <c r="A21" t="s">
         <v>11</v>
       </c>
@@ -712,7 +743,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:2">
       <c r="A22" t="s">
         <v>12</v>
       </c>
@@ -720,7 +751,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:2">
       <c r="A23" t="s">
         <v>13</v>
       </c>
@@ -728,8 +759,42 @@
         <v>45</v>
       </c>
     </row>
+    <row r="24" spans="1:2">
+      <c r="A24" t="s">
+        <v>63</v>
+      </c>
+      <c r="B24" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="15">
+      <c r="A27" s="3" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="A29" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="A31" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2">
+      <c r="A32" t="s">
+        <v>70</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;C&amp;"Calibri"&amp;10&amp;K000000 IN-CONFIDENCE&amp;1#_x000D_</oddHeader>
   </headerFooter>
@@ -738,13 +803,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{838DC91F-E55C-4C6C-BCAE-AE41EA2C8CC0}">
-  <dimension ref="A1:N10"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:O11"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="14" width="12.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -787,8 +852,11 @@
       <c r="N1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -798,8 +866,11 @@
       <c r="E2" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="O2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -831,7 +902,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -842,84 +913,92 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15">
       <c r="A5" t="s">
+        <v>62</v>
+      </c>
+      <c r="I5" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15">
+      <c r="A6" t="s">
         <v>26</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I6" t="s">
         <v>27</v>
       </c>
-      <c r="J5" t="s">
+      <c r="J6" t="s">
         <v>28</v>
       </c>
-      <c r="K5" t="s">
+      <c r="K6" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>30</v>
-      </c>
-      <c r="I6" t="s">
-        <v>31</v>
-      </c>
-      <c r="J6" t="s">
-        <v>32</v>
-      </c>
-      <c r="K6" t="s">
-        <v>33</v>
-      </c>
-      <c r="L6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15">
       <c r="A7" t="s">
         <v>30</v>
       </c>
+      <c r="I7" t="s">
+        <v>31</v>
+      </c>
+      <c r="J7" t="s">
+        <v>32</v>
+      </c>
+      <c r="K7" t="s">
+        <v>33</v>
+      </c>
       <c r="L7" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15">
       <c r="A8" t="s">
         <v>30</v>
       </c>
       <c r="L8" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15">
       <c r="A9" t="s">
         <v>30</v>
       </c>
-      <c r="I9" t="s">
-        <v>37</v>
-      </c>
-      <c r="J9" t="s">
-        <v>37</v>
-      </c>
-      <c r="K9" t="s">
-        <v>37</v>
-      </c>
       <c r="L9" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15">
       <c r="A10" t="s">
         <v>30</v>
       </c>
       <c r="I10" t="s">
+        <v>37</v>
+      </c>
+      <c r="J10" t="s">
+        <v>37</v>
+      </c>
+      <c r="K10" t="s">
+        <v>37</v>
+      </c>
+      <c r="L10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15">
+      <c r="A11" t="s">
+        <v>30</v>
+      </c>
+      <c r="I11" t="s">
         <v>38</v>
       </c>
-      <c r="J10" t="s">
+      <c r="J11" t="s">
         <v>38</v>
       </c>
-      <c r="K10" t="s">
+      <c r="K11" t="s">
         <v>38</v>
       </c>
-      <c r="L10" t="s">
+      <c r="L11" t="s">
         <v>38</v>
       </c>
     </row>

</xml_diff>